<commit_message>
docs: gate_fit sheet — 5 variables for the decoder pixel-class gate; 9-way REFUSED, 4-way cost-tier SUPPORTED (LOCO-CV 0.804)
P2 fit under the gate_refit laws: dispatch-time-observable inputs only,
leave-one-CLIP-out validation. 9-way fine classification refused (train
0.922 vs CV 0.157 — ~2 clips/class is fitting on one point). The 4-way
cost-tier gate holds: ENTROPY-EXTREME / DENSE-INTER / MID / LIGHT, train
1.000, CV 0.804 across 17 clip-folds. Variables: entropy_calls_per_mb,
mb_skip_frac, bits_per_mb, skiprecon_calls_per_mb, dequant_calls_per_mb.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/big-oppy-decoder-truthtable.xlsx
+++ b/docs/big-oppy-decoder-truthtable.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="method" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="truth_table" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="class_summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gate_fit" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -441,7 +442,6 @@
           <t>decoder pixel-class truth table</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -7580,4 +7580,685 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C63"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>decoder pixel-class gate fit (P2) — greedy tree, &lt;=5 dispatch-time variables, leave-one-CLIP-out validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>VERDICT</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>9-way fine classes</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>REFUSED: train 0.922 vs LOCO-CV 0.157 — ~2 clips/class cannot support a 9-way gate (gate_refit law 3: fitting on one point)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>4-way cost tiers</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SUPPORTED: train 1.000, LOCO-CV 0.804 over 51 rows / 17 clip-folds</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>superclasses</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ENTROPY-EXTREME={grain}  DENSE-INTER={fastmotion,detail,pan,complex}  MID={medium,smooth}  LIGHT={screen,static}</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>caveat</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>valid on varied axes only: class x tier x resolution, qp26, x264 provenance. NOT validated across qp/bitrate/other encoders</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>selected variables, 4-way gate (order of first use)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>entropy_calls_per_mb</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>mb_skip_frac</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>3</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>bits_per_mb</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>4</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>skiprecon_calls_per_mb</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>5</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>dequant_calls_per_mb</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>4-way decision tree (thresholds)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>entropy_calls_per_mb &lt;= 2.565?</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  mb_skip_frac &lt;= 0.157?</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    -&gt; MID</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  mb_skip_frac &gt; 0.157:</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    -&gt; LIGHT</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>entropy_calls_per_mb &gt; 2.565:</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  bits_per_mb &lt;= 363.665?</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    skiprecon_calls_per_mb &lt;= 0.494?</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      dequant_calls_per_mb &lt;= 1.92?</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        -&gt; MID</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      dequant_calls_per_mb &gt; 1.92:</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        -&gt; DENSE-INTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    skiprecon_calls_per_mb &gt; 0.494:</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      -&gt; MID</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  bits_per_mb &gt; 363.665:</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    -&gt; ENTROPY-EXTREME</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>single-feature ranking (4-way)</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>info gain</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>1-feature acc</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>entropy_calls_per_mb</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>0.7433999999999999</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0.922</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>dequant_calls_per_mb</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>0.6589</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>bits_per_mb</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>0.5832000000000001</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0.961</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>mb_intra_frac</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>0.5226</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0.922</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>skiprecon_calls_per_mb</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>0.5226</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0.922</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>intra_calls_per_mb</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>0.432</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0.804</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>mb_skip_frac</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0.922</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>mb_p_frac</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>0.3591</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0.765</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>mc_calls_per_mb</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>0.2886</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0.824</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>mbs_per_frame</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>0.1539</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0.471</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>mb_b_frac</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>0.0431</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0.569</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>is_cabac</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0.471</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>4-way CV confusion: true</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>correct/total</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>misses</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>DENSE-INTER</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>23/24</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>{'MID': 1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>ENTROPY-EXTREME</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>4/6</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>{'DENSE-INTER': 2}</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>LIGHT</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>9/12</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>{'MID': 2, 'DENSE-INTER': 1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>5/9</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>{'LIGHT': 2, 'DENSE-INTER': 2}</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>9-way CV confusion (the refusal evidence): true</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>correct/total</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>misses</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>complex</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>0/6</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>{'screen': 1, 'pan': 4, 'detail': 1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>detail</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>0/6</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>{'complex': 2, 'pan': 2, 'fastmotion': 2}</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>fastmotion</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>0/6</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>{'pan': 5, 'complex': 1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>grain</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>6/6</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2/6</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>{'complex': 2, 'detail': 1, 'static': 1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>pan</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>0/6</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>{'complex': 4, 'detail': 2}</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>screen</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>0/6</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>{'static': 3, 'complex': 1, 'medium': 2}</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>smooth</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>0/3</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>{'medium': 1, 'screen': 2}</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>0/6</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>{'screen': 6}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: per-tier gate-fit verdict — variables tier-stable, thresholds swing 2.4x, wire per-tier behind GATE 0; cavlc mb-frac columns flagged INVALID (CABAC-only scopes)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/big-oppy-decoder-truthtable.xlsx
+++ b/docs/big-oppy-decoder-truthtable.xlsx
@@ -7588,7 +7588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:C69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -8171,7 +8171,6 @@
           <t>6/6</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -8255,6 +8254,61 @@
       <c r="C63" t="inlineStr">
         <is>
           <t>{'screen': 6}</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="inlineStr">
+        <is>
+          <t>PER-TIER FIT (are the fittings identical across tool tiers?)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>variables + tree SHAPE tier-stable; THRESHOLDS are not — root entropy_calls_per_mb: cavlc 5.575 / main 3.575 / high 2.335 (2.4x swing; the feature measures different call structures per coder). bits_per_mb split: 406.7 / 315.4 / 340.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>pooled tree CV by tier</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>cavlc 0.882, main 0.765, high 0.765 — pooled is a fair compromise, but wiring should use PER-TIER thresholds behind GATE 0 (tool tier routes first anyway)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>per-tier independent fits</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>cavlc train 1.000 CV 0.824; main train 1.000 CV 0.765; high train 1.000 CV 0.765 (17 rows each — small-N, verdict rests on 17 clip-folds)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>DATA DEFECT (found via impossible number)</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>mb_skip_frac median 0.948 on cavlc tier: dec-mb-P/B scopes exist only in the CABAC loop, so mb_p_frac/mb_b_frac read 0 and skip_frac ~= 1 - intra on ALL cavlc rows. mb_p/b/skip fracs are INVALID on the cavlc tier; pooled tree survives because cavlc routes on entropy_calls first. Fix: add CAVLC-loop MB scopes before wiring skip_frac into any cavlc-tier gate</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: GATE 1 full per-tier fittings — 3-variable core, per-tier thresholds; cavlc fit excludes its invalid columns
cavlc train 1.000 CV 0.824 (entropy_calls x2 + bits_per_mb); main 1.000/0.765
and high 1.000/0.824 (entropy_calls + skiprecon + bits_per_mb — skiprecon
replaced the CABAC-only mb_skip_frac and IMPROVED high's CV). DENSE-INTER
23/24, ENTROPY-EXTREME 6/6; weakest cell MID-on-main 0/3. Sheet
gate_fit_per_tier carries trees, rankings, confusions, small-N notice.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/big-oppy-decoder-truthtable.xlsx
+++ b/docs/big-oppy-decoder-truthtable.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="truth_table" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="class_summary" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gate_fit" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gate_fit_per_tier" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8315,4 +8316,1051 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C96"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>GATE 1 — full per-tier fittings (4-way cost-tier superclasses)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>method</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>same P2 fitter as gate_fit, run per tool tier; cavlc EXCLUDES mb_p/b/skip_frac (CABAC-only scopes — invalid columns on that tier); min-leaf 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>small-N notice</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>17 rows / 17 clip-folds per tier — each verdict rests on &lt;=6 clips per superclass; treat thresholds as v1, refit after qp sweep</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1">
+        <f>== CAVLC ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>train / LOCO-CV</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1.000 / 0.824 (17 rows, 17 folds)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>variables (order of first use)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>entropy_calls_per_mb, bits_per_mb</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>tree</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>entropy_calls_per_mb &lt;= 5.575?</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  entropy_calls_per_mb &lt;= 2.96?</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    -&gt; LIGHT</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  entropy_calls_per_mb &gt; 2.96:</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    -&gt; MID</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>entropy_calls_per_mb &gt; 5.575:</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  bits_per_mb &lt;= 406.65?</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    -&gt; DENSE-INTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  bits_per_mb &gt; 406.65:</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    -&gt; ENTROPY-EXTREME</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>single-feature ranking</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>info gain</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>1-feature acc</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>entropy_calls_per_mb</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.9774</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>dequant_calls_per_mb</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.9774</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>skiprecon_calls_per_mb</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0.9774</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>mc_calls_per_mb</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>0.8355</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>bits_per_mb</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0.7458</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>mb_intra_frac</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0.5226</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.824</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>intra_calls_per_mb</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>0.4165</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.706</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>mbs_per_frame</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0.1539</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.471</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>CV confusion: true</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>correct/total</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>misses</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>DENSE-INTER</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>7/8</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>{'MID': 1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>ENTROPY-EXTREME</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2/2</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>LIGHT</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>{'DENSE-INTER': 1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2/3</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>{'DENSE-INTER': 1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1">
+        <f>== MAIN ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>train / LOCO-CV</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1.000 / 0.765 (17 rows, 17 folds)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>variables (order of first use)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>entropy_calls_per_mb, skiprecon_calls_per_mb, bits_per_mb</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>tree</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>entropy_calls_per_mb &lt;= 3.575?</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  skiprecon_calls_per_mb &lt;= 0.32?</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    -&gt; MID</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  skiprecon_calls_per_mb &gt; 0.32:</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    -&gt; LIGHT</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>entropy_calls_per_mb &gt; 3.575:</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  bits_per_mb &lt;= 315.43?</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    -&gt; DENSE-INTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  bits_per_mb &gt; 315.43:</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    -&gt; ENTROPY-EXTREME</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>single-feature ranking</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>info gain</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>1-feature acc</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>entropy_calls_per_mb</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>0.9774</v>
+      </c>
+      <c r="C49" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>dequant_calls_per_mb</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>0.9774</v>
+      </c>
+      <c r="C50" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>mb_p_frac</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>0.9367</v>
+      </c>
+      <c r="C51" t="n">
+        <v>0.882</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>skiprecon_calls_per_mb</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>0.7871</v>
+      </c>
+      <c r="C52" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>mb_skip_frac</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>0.7871</v>
+      </c>
+      <c r="C53" t="n">
+        <v>0.882</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>bits_per_mb</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>0.5283</v>
+      </c>
+      <c r="C54" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>mb_intra_frac</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>0.5226</v>
+      </c>
+      <c r="C55" t="n">
+        <v>0.882</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>intra_calls_per_mb</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>0.5226</v>
+      </c>
+      <c r="C56" t="n">
+        <v>0.824</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>mc_calls_per_mb</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>0.3165</v>
+      </c>
+      <c r="C57" t="n">
+        <v>0.882</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>mb_b_frac</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>0.2271</v>
+      </c>
+      <c r="C58" t="n">
+        <v>0.647</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>mbs_per_frame</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>0.1539</v>
+      </c>
+      <c r="C59" t="n">
+        <v>0.471</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>CV confusion: true</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>correct/total</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>misses</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>DENSE-INTER</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>8/8</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>ENTROPY-EXTREME</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2/2</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>LIGHT</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>{'MID': 1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>0/3</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>{'LIGHT': 3}</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1">
+        <f>== HIGH ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>train / LOCO-CV</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>1.000 / 0.824 (17 rows, 17 folds)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>variables (order of first use)</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>entropy_calls_per_mb, skiprecon_calls_per_mb, bits_per_mb</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="inlineStr">
+        <is>
+          <t>tree</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>entropy_calls_per_mb &lt;= 2.335?</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  skiprecon_calls_per_mb &lt;= 0.3575?</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    -&gt; MID</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  skiprecon_calls_per_mb &gt; 0.3575:</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    -&gt; LIGHT</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>entropy_calls_per_mb &gt; 2.335:</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  bits_per_mb &lt;= 340.11?</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    -&gt; DENSE-INTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  bits_per_mb &gt; 340.11:</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    -&gt; ENTROPY-EXTREME</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>single-feature ranking</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>info gain</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>1-feature acc</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>entropy_calls_per_mb</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>0.9774</v>
+      </c>
+      <c r="C81" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>dequant_calls_per_mb</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>0.9774</v>
+      </c>
+      <c r="C82" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>mb_p_frac</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>0.8355</v>
+      </c>
+      <c r="C83" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>skiprecon_calls_per_mb</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>0.7871</v>
+      </c>
+      <c r="C84" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>mb_skip_frac</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>0.7871</v>
+      </c>
+      <c r="C85" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>bits_per_mb</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>0.7458</v>
+      </c>
+      <c r="C86" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>intra_calls_per_mb</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>0.6157</v>
+      </c>
+      <c r="C87" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>mb_intra_frac</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>0.5283</v>
+      </c>
+      <c r="C88" t="n">
+        <v>0.824</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>mc_calls_per_mb</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>0.5102</v>
+      </c>
+      <c r="C89" t="n">
+        <v>0.706</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>mb_b_frac</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>0.2857</v>
+      </c>
+      <c r="C90" t="n">
+        <v>0.647</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>mbs_per_frame</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>0.1539</v>
+      </c>
+      <c r="C91" t="n">
+        <v>0.471</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>CV confusion: true</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>correct/total</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>misses</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>DENSE-INTER</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>8/8</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>ENTROPY-EXTREME</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2/2</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>LIGHT</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>{'DENSE-INTER': 1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>1/3</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>{'LIGHT': 1, 'DENSE-INTER': 1}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: sec 6 MAIN — per-class competitive gap vs ffmpeg on default streams (grain 1.5x .. static 3.2x); LIGHT content named worst class (per-frame overhead, not kernels)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/big-oppy-decoder-truthtable.xlsx
+++ b/docs/big-oppy-decoder-truthtable.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gate_fit" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gate_fit_per_tier" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="main_vs_default" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="vs_ffmpeg_default" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -14409,4 +14410,409 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ours vs ffmpeg, SAME x264-default streams; concat &gt;=800ms, frames verified, best-of-3 alternating; loaded box — ratio robust</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>class</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>clip</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>ours ns/MB</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>ffmpeg ns/MB</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>gap</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>FourPeople_1280x720_60</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>890</v>
+      </c>
+      <c r="D3" t="n">
+        <v>289</v>
+      </c>
+      <c r="E3" t="n">
+        <v>3.08</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>static</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>akiyo_cif</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>878</v>
+      </c>
+      <c r="D4" t="n">
+        <v>267</v>
+      </c>
+      <c r="E4" t="n">
+        <v>3.29</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>foreman_cif</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1681</v>
+      </c>
+      <c r="D5" t="n">
+        <v>804</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2.09</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>in_to_tree_420_720p50</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1431</v>
+      </c>
+      <c r="D6" t="n">
+        <v>603</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2.37</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>detail</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>720p50_shields_ter</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1669</v>
+      </c>
+      <c r="D7" t="n">
+        <v>796</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>detail</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>mobile_cif</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>3309</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1776</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1.86</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>pan</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>720p5994_stockholm_ter</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1733</v>
+      </c>
+      <c r="D9" t="n">
+        <v>819</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2.11</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>pan</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>bus_cif</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2830</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1536</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1.84</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>complex</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>crew_4cif</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1705</v>
+      </c>
+      <c r="D11" t="n">
+        <v>768</v>
+      </c>
+      <c r="E11" t="n">
+        <v>2.22</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>complex</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>tempete_cif</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2758</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1424</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1.94</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>fastmotion</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>crowd_run_1080p50</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>3057</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1565</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1.95</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>fastmotion</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>football_cif</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>3111</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1698</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1.83</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>smooth</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>blue_sky_1080p25</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1343</v>
+      </c>
+      <c r="D15" t="n">
+        <v>559</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>grain</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>grain_akiyo</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>7462</v>
+      </c>
+      <c r="D16" t="n">
+        <v>4935</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1.51</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>grain</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>grain_flat</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>7292</v>
+      </c>
+      <c r="D17" t="n">
+        <v>5126</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1.42</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>screen</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>screen_text</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>631</v>
+      </c>
+      <c r="D18" t="n">
+        <v>227</v>
+      </c>
+      <c r="E18" t="n">
+        <v>2.78</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>screen</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>screen_ui</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1448</v>
+      </c>
+      <c r="D19" t="n">
+        <v>686</v>
+      </c>
+      <c r="E19" t="n">
+        <v>2.11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>